<commit_message>
Fix Calificaciones_Web1.xlsx: rutas OPC con forward-slash para compatibilidad con Office
</commit_message>
<xml_diff>
--- a/Web 1/Calificaciones_Web1.xlsx
+++ b/Web 1/Calificaciones_Web1.xlsx
@@ -1,5 +1,13 @@
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Calificaciones" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="4">
     <font>
@@ -65,15 +73,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="Calificaciones" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Mejora Calificaciones_Web1.xlsx: anchos de columna y DEFINITIVA como numero
</commit_message>
<xml_diff>
--- a/Web 1/Calificaciones_Web1.xlsx
+++ b/Web 1/Calificaciones_Web1.xlsx
@@ -75,6 +75,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="55" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
@@ -247,7 +254,7 @@
         <v>3.7</v>
       </c>
       <c r="H5" t="n" s="3">
-        <v>3,3</v>
+        <v>3.3</v>
       </c>
       <c r="I5" t="inlineStr" s="0">
         <is>
@@ -282,7 +289,7 @@
         <v>4.0</v>
       </c>
       <c r="H6" t="n" s="3">
-        <v>4,5</v>
+        <v>4.5</v>
       </c>
       <c r="I6" t="inlineStr" s="0">
         <is>
@@ -317,7 +324,7 @@
         <v>2.8</v>
       </c>
       <c r="H7" t="n" s="3">
-        <v>3,5</v>
+        <v>3.5</v>
       </c>
       <c r="I7" t="inlineStr" s="0">
         <is>
@@ -352,7 +359,7 @@
         <v>0.0</v>
       </c>
       <c r="H8" t="n" s="3">
-        <v>2,6</v>
+        <v>2.6</v>
       </c>
       <c r="I8" t="inlineStr" s="0">
         <is>
@@ -387,7 +394,7 @@
         <v>0.0</v>
       </c>
       <c r="H9" t="n" s="3">
-        <v>2,5</v>
+        <v>2.5</v>
       </c>
       <c r="I9" t="inlineStr" s="0">
         <is>
@@ -424,7 +431,7 @@
         <v>4.3</v>
       </c>
       <c r="H10" t="n" s="3">
-        <v>3,8</v>
+        <v>3.8</v>
       </c>
       <c r="I10" t="inlineStr" s="0">
         <is>
@@ -461,7 +468,7 @@
         <v>3.0</v>
       </c>
       <c r="H11" t="n" s="3">
-        <v>2,6</v>
+        <v>2.6</v>
       </c>
       <c r="I11" t="inlineStr" s="0">
         <is>
@@ -502,7 +509,7 @@
         <v>0.0</v>
       </c>
       <c r="H12" t="n" s="3">
-        <v>0,7</v>
+        <v>0.7</v>
       </c>
       <c r="I12" t="inlineStr" s="0">
         <is>
@@ -543,7 +550,7 @@
         <v>0.0</v>
       </c>
       <c r="H13" t="n" s="3">
-        <v>0,8</v>
+        <v>0.8</v>
       </c>
       <c r="I13" t="inlineStr" s="0">
         <is>
@@ -582,7 +589,7 @@
         <v>0.5</v>
       </c>
       <c r="H14" t="n" s="3">
-        <v>1,5</v>
+        <v>1.5</v>
       </c>
       <c r="I14" t="inlineStr" s="0">
         <is>
@@ -623,7 +630,7 @@
         <v>3.8</v>
       </c>
       <c r="H15" t="n" s="3">
-        <v>1,4</v>
+        <v>1.4</v>
       </c>
       <c r="I15" t="inlineStr" s="0">
         <is>
@@ -664,7 +671,7 @@
         <v>0.0</v>
       </c>
       <c r="H16" t="n" s="3">
-        <v>0,6</v>
+        <v>0.6</v>
       </c>
       <c r="I16" t="inlineStr" s="0">
         <is>
@@ -699,7 +706,7 @@
         <v>3.8</v>
       </c>
       <c r="H17" t="n" s="3">
-        <v>3,7</v>
+        <v>3.7</v>
       </c>
       <c r="I17" t="inlineStr" s="0">
         <is>
@@ -734,7 +741,7 @@
         <v>4.2</v>
       </c>
       <c r="H18" t="n" s="3">
-        <v>3,4</v>
+        <v>3.4</v>
       </c>
       <c r="I18" t="inlineStr" s="0">
         <is>
@@ -769,7 +776,7 @@
         <v>2.8</v>
       </c>
       <c r="H19" t="n" s="3">
-        <v>3,2</v>
+        <v>3.2</v>
       </c>
       <c r="I19" t="inlineStr" s="0">
         <is>
@@ -804,7 +811,7 @@
         <v>3.6</v>
       </c>
       <c r="H20" t="n" s="3">
-        <v>3,4</v>
+        <v>3.4</v>
       </c>
       <c r="I20" t="inlineStr" s="0">
         <is>
@@ -841,7 +848,7 @@
         <v>3.3</v>
       </c>
       <c r="H21" t="n" s="3">
-        <v>3,3</v>
+        <v>3.3</v>
       </c>
       <c r="I21" t="inlineStr" s="0">
         <is>
@@ -878,7 +885,7 @@
         <v>5.0</v>
       </c>
       <c r="H22" t="n" s="3">
-        <v>3,7</v>
+        <v>3.7</v>
       </c>
       <c r="I22" t="inlineStr" s="0">
         <is>
@@ -915,7 +922,7 @@
         </is>
       </c>
       <c r="H23" t="n" s="3">
-        <v>2,8</v>
+        <v>2.8</v>
       </c>
       <c r="I23" t="inlineStr" s="0">
         <is>

</xml_diff>